<commit_message>
update 6 quan trong
</commit_message>
<xml_diff>
--- a/Dice_Jobs_Final.xlsx
+++ b/Dice_Jobs_Final.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,16 +427,16 @@
         <v>Easy Apply</v>
       </c>
       <c r="B2" t="str">
-        <v>N/A</v>
+        <v>US Postal Service</v>
       </c>
       <c r="C2" t="str">
-        <v>354-291</v>
+        <v>78160 - 144820</v>
       </c>
       <c r="D2" t="str">
-        <v>N/A</v>
+        <v>Atlanta, Georgia</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>2d ago</v>
       </c>
       <c r="F2" t="str">
         <v>https://www.dice.com/job-detail/51e13a7e-1e2a-475d-bda3-82172c070e1b</v>
@@ -450,16 +450,16 @@
         <v>Forensic Computer Analyst</v>
       </c>
       <c r="B3" t="str">
-        <v>N/A</v>
+        <v>US Postal Service</v>
       </c>
       <c r="C3" t="str">
-        <v>354-291</v>
+        <v>78160 - 144820</v>
       </c>
       <c r="D3" t="str">
-        <v>N/A</v>
+        <v>Atlanta, Georgia</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>2d ago</v>
       </c>
       <c r="F3" t="str">
         <v>https://www.dice.com/job-detail/51e13a7e-1e2a-475d-bda3-82172c070e1b</v>
@@ -473,16 +473,16 @@
         <v>Easy Apply</v>
       </c>
       <c r="B4" t="str">
-        <v>N/A</v>
+        <v>Infinite Computer Solutions (ICS)</v>
       </c>
       <c r="C4" t="str">
         <v>$80,000 - $90,000</v>
       </c>
       <c r="D4" t="str">
-        <v>N/A</v>
+        <v>Berkeley Heights, New Jersey</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>Yesterday</v>
       </c>
       <c r="F4" t="str">
         <v>https://www.dice.com/job-detail/68408ed2-b49c-4d41-9138-dcae74f77e65</v>
@@ -493,25 +493,25 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Certified Financial Planner, Tax Channel</v>
+        <v>Implementation Analyst (Banking Experience Required)</v>
       </c>
       <c r="B5" t="str">
-        <v>N/A</v>
+        <v>Infinite Computer Solutions (ICS)</v>
       </c>
       <c r="C5" t="str">
-        <v>00 - 110</v>
+        <v>$80,000 - $90,000</v>
       </c>
       <c r="D5" t="str">
-        <v>N/A</v>
+        <v>Berkeley Heights, New Jersey</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>Yesterday</v>
       </c>
       <c r="F5" t="str">
-        <v>https://www.dice.com/job-detail/dbbb83dd-102b-4e4e-9238-44f0885b0636</v>
+        <v>https://www.dice.com/job-detail/68408ed2-b49c-4d41-9138-dcae74f77e65</v>
       </c>
       <c r="G5" t="str">
-        <v>CFA</v>
+        <v>Analyst</v>
       </c>
     </row>
     <row r="6">
@@ -519,45 +519,45 @@
         <v>Easy Apply</v>
       </c>
       <c r="B6" t="str">
-        <v>N/A</v>
+        <v>Strategic Staffing Solutions</v>
       </c>
       <c r="C6" t="str">
-        <v>$70 - $80</v>
+        <v>USD0</v>
       </c>
       <c r="D6" t="str">
-        <v>N/A</v>
+        <v>Charlotte, North Carolina</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>Today</v>
       </c>
       <c r="F6" t="str">
-        <v>https://www.dice.com/job-detail/ee5e0eb9-0a34-4cd5-8c21-36f37e666d90</v>
+        <v>https://www.dice.com/job-detail/6af22463-0d9b-4d22-8c20-ff44c1200086</v>
       </c>
       <c r="G6" t="str">
-        <v>CFA</v>
+        <v>Analyst</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Sr. Business Analyst/Product Owner - UI/UX</v>
+        <v>Application Analyst (Python / PyFlink / Data Engineering)</v>
       </c>
       <c r="B7" t="str">
-        <v>N/A</v>
+        <v>Strategic Staffing Solutions</v>
       </c>
       <c r="C7" t="str">
-        <v>$70 - $80</v>
+        <v>USD0</v>
       </c>
       <c r="D7" t="str">
-        <v>N/A</v>
+        <v>Charlotte, North Carolina</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>Today</v>
       </c>
       <c r="F7" t="str">
-        <v>https://www.dice.com/job-detail/ee5e0eb9-0a34-4cd5-8c21-36f37e666d90</v>
+        <v>https://www.dice.com/job-detail/6af22463-0d9b-4d22-8c20-ff44c1200086</v>
       </c>
       <c r="G7" t="str">
-        <v>CFA</v>
+        <v>Analyst</v>
       </c>
     </row>
     <row r="8">
@@ -565,211 +565,487 @@
         <v>Easy Apply</v>
       </c>
       <c r="B8" t="str">
-        <v>N/A</v>
+        <v>Bright Sol</v>
       </c>
       <c r="C8" t="str">
-        <v>45-50</v>
+        <v>60 - 65</v>
       </c>
       <c r="D8" t="str">
-        <v>N/A</v>
+        <v>Sacramento, California</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>Today</v>
       </c>
       <c r="F8" t="str">
-        <v>https://www.dice.com/job-detail/a429546e-1e5e-4820-a86e-b586c5c09f37</v>
+        <v>https://www.dice.com/job-detail/6b0b7ed6-7d41-4cfe-ae2e-24756c06ff07</v>
       </c>
       <c r="G8" t="str">
-        <v>CEO</v>
+        <v>CFA</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Executive IT Services Specialist</v>
+        <v>Financial Services Manager</v>
       </c>
       <c r="B9" t="str">
-        <v>N/A</v>
+        <v>Bright Sol</v>
       </c>
       <c r="C9" t="str">
-        <v>45-50</v>
+        <v>60 - 65</v>
       </c>
       <c r="D9" t="str">
-        <v>N/A</v>
+        <v>Sacramento, California</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>Today</v>
       </c>
       <c r="F9" t="str">
-        <v>https://www.dice.com/job-detail/a429546e-1e5e-4820-a86e-b586c5c09f37</v>
+        <v>https://www.dice.com/job-detail/6b0b7ed6-7d41-4cfe-ae2e-24756c06ff07</v>
       </c>
       <c r="G9" t="str">
-        <v>CEO</v>
+        <v>CFA</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Easy Apply</v>
+        <v>Certified Financial Planner, Tax Channel</v>
       </c>
       <c r="B10" t="str">
-        <v>N/A</v>
+        <v>Cetera Financial Group, Inc.</v>
       </c>
       <c r="C10" t="str">
-        <v>$75000</v>
+        <v>USD 90</v>
       </c>
       <c r="D10" t="str">
-        <v>N/A</v>
+        <v>Dallas, Texas</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>Today</v>
       </c>
       <c r="F10" t="str">
-        <v>https://www.dice.com/job-detail/b2333592-3ab7-4ac0-ad65-17215525dd15</v>
+        <v>https://www.dice.com/job-detail/dbbb83dd-102b-4e4e-9238-44f0885b0636</v>
       </c>
       <c r="G10" t="str">
-        <v>CEO</v>
+        <v>CFA</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>IT Applications Engineer V - Data Science, Data &amp; AI Engineering, Application Engineering</v>
+        <v>Easy Apply</v>
       </c>
       <c r="B11" t="str">
-        <v>N/A</v>
+        <v>Xoriant Corporation</v>
       </c>
       <c r="C11" t="str">
-        <v>00 - 204</v>
+        <v>$70 - $80</v>
       </c>
       <c r="D11" t="str">
-        <v>N/A</v>
+        <v>Hybrid in New York, New York</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>10d ago</v>
       </c>
       <c r="F11" t="str">
-        <v>https://www.dice.com/job-detail/ffe21eeb-b255-4368-8e62-0b2896c692d3</v>
+        <v>https://www.dice.com/job-detail/ee5e0eb9-0a34-4cd5-8c21-36f37e666d90</v>
       </c>
       <c r="G11" t="str">
-        <v>Data Science</v>
+        <v>CFA</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>FLEX Manager, Data Science - Pricing Models</v>
+        <v>Sr. Business Analyst/Product Owner - UI/UX</v>
       </c>
       <c r="B12" t="str">
-        <v>N/A</v>
+        <v>Xoriant Corporation</v>
       </c>
       <c r="C12" t="str">
-        <v>73 - 51</v>
+        <v>$70 - $80</v>
       </c>
       <c r="D12" t="str">
-        <v>N/A</v>
+        <v>Hybrid in New York, New York</v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>10d ago</v>
       </c>
       <c r="F12" t="str">
-        <v>https://www.dice.com/job-detail/7b3f5f72-92c5-4b09-8bfe-24b119610617</v>
+        <v>https://www.dice.com/job-detail/ee5e0eb9-0a34-4cd5-8c21-36f37e666d90</v>
       </c>
       <c r="G12" t="str">
-        <v>Data Science</v>
+        <v>CFA</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Senior Platform Engineer- Data Science</v>
+        <v>Equity Strategist</v>
       </c>
       <c r="B13" t="str">
-        <v>N/A</v>
+        <v>UBS</v>
       </c>
       <c r="C13" t="str">
-        <v>00 - 68</v>
+        <v>USD 145</v>
       </c>
       <c r="D13" t="str">
-        <v>N/A</v>
+        <v>New York, New York</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>3d ago</v>
       </c>
       <c r="F13" t="str">
-        <v>https://www.dice.com/job-detail/2ba26ebe-8e39-4bba-9266-be9c1177827f</v>
+        <v>https://www.dice.com/job-detail/b5008b16-720e-4729-a54a-2e9bbeef4ccf</v>
       </c>
       <c r="G13" t="str">
-        <v>Data Science</v>
+        <v>CFA</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Easy Apply</v>
+        <v>Hair Stylist/Barber</v>
       </c>
       <c r="B14" t="str">
-        <v>N/A</v>
+        <v>Sport Clips</v>
       </c>
       <c r="C14" t="str">
-        <v>$110000</v>
+        <v>USD 25</v>
       </c>
       <c r="D14" t="str">
-        <v>N/A</v>
+        <v>Danvers, Massachusetts</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>30+d ago</v>
       </c>
       <c r="F14" t="str">
-        <v>https://www.dice.com/job-detail/c8cbc56c-9d36-4dfc-b67f-9785ccc187b5</v>
+        <v>https://www.dice.com/job-detail/0f465078-3ac3-4862-93e5-1a229fe0c9ae</v>
       </c>
       <c r="G14" t="str">
-        <v>FP&amp;A</v>
+        <v>CEO</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SR FP&amp;A Analyst</v>
+        <v>Easy Apply</v>
       </c>
       <c r="B15" t="str">
-        <v>N/A</v>
+        <v>InfoPeople Corp</v>
       </c>
       <c r="C15" t="str">
-        <v>$110000</v>
+        <v>$140,000 - $180,000</v>
       </c>
       <c r="D15" t="str">
-        <v>N/A</v>
+        <v>Remote</v>
       </c>
       <c r="E15" t="str">
-        <v/>
+        <v>14d ago</v>
       </c>
       <c r="F15" t="str">
-        <v>https://www.dice.com/job-detail/c8cbc56c-9d36-4dfc-b67f-9785ccc187b5</v>
+        <v>https://www.dice.com/job-detail/bded6ae6-06af-41e8-8279-f67819b5564c</v>
       </c>
       <c r="G15" t="str">
-        <v>FP&amp;A</v>
+        <v>CEO</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
+        <v>VP of Operations</v>
+      </c>
+      <c r="B16" t="str">
+        <v>InfoPeople Corp</v>
+      </c>
+      <c r="C16" t="str">
+        <v>$140,000 - $180,000</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="E16" t="str">
+        <v>14d ago</v>
+      </c>
+      <c r="F16" t="str">
+        <v>https://www.dice.com/job-detail/bded6ae6-06af-41e8-8279-f67819b5564c</v>
+      </c>
+      <c r="G16" t="str">
+        <v>CEO</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>IT Applications Engineer V - Data Science, Data &amp; AI Engineering, Application Engineering</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Kaiser Permanente</v>
+      </c>
+      <c r="C17" t="str">
+        <v>USD 158</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Pleasanton, California</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Today</v>
+      </c>
+      <c r="F17" t="str">
+        <v>https://www.dice.com/job-detail/ffe21eeb-b255-4368-8e62-0b2896c692d3</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Data Science</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Senior Platform Engineer- Data Science</v>
+      </c>
+      <c r="B18" t="str">
+        <v>TEKsystems c/o Allegis Group</v>
+      </c>
+      <c r="C18" t="str">
+        <v>USD 55</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Columbus, Ohio</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Today</v>
+      </c>
+      <c r="F18" t="str">
+        <v>https://www.dice.com/job-detail/940d7c94-7721-473d-bb71-0143fa825610</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Data Science</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Geo / Earth Data Science Internship</v>
+      </c>
+      <c r="B19" t="str">
+        <v>SAIC</v>
+      </c>
+      <c r="C19" t="str">
+        <v>026-04</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Reston, Virginia</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Today</v>
+      </c>
+      <c r="F19" t="str">
+        <v>https://www.dice.com/job-detail/34158c1c-b2b7-4dd5-96d3-2e6f5dd44cef</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Data Science</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
         <v>Easy Apply</v>
       </c>
-      <c r="B16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="C16" t="str">
+      <c r="B20" t="str">
+        <v>Motion Recruitment Partners, LLC</v>
+      </c>
+      <c r="C20" t="str">
+        <v>$50 - $70</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Los Angeles, California</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Today</v>
+      </c>
+      <c r="F20" t="str">
+        <v>https://www.dice.com/job-detail/1201c12a-4c76-4101-8a5d-ee06514f5c84</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Data Science</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Data Science Engineer / Los Angeles / Fully Onsite / Python / LLMs / MongoDB</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Motion Recruitment Partners, LLC</v>
+      </c>
+      <c r="C21" t="str">
+        <v>$50 - $70</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Los Angeles, California</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Today</v>
+      </c>
+      <c r="F21" t="str">
+        <v>https://www.dice.com/job-detail/1201c12a-4c76-4101-8a5d-ee06514f5c84</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Data Science</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Senior Analyst, Data Science and Analytics</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Trans Union LLC</v>
+      </c>
+      <c r="C22" t="str">
+        <v>USD 67</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Chicago, Illinois</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Today</v>
+      </c>
+      <c r="F22" t="str">
+        <v>https://www.dice.com/job-detail/ac757413-35b9-44cf-a01b-d4853c1ed5f0</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Data Science</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Easy Apply</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Dexian DISYS</v>
+      </c>
+      <c r="C23" t="str">
+        <v>$110</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Tampa, Florida</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Today</v>
+      </c>
+      <c r="F23" t="str">
+        <v>https://www.dice.com/job-detail/c8cbc56c-9d36-4dfc-b67f-9785ccc187b5</v>
+      </c>
+      <c r="G23" t="str">
+        <v>FP&amp;A</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>SR FP&amp;A Analyst</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Dexian DISYS</v>
+      </c>
+      <c r="C24" t="str">
+        <v>$110</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Tampa, Florida</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Today</v>
+      </c>
+      <c r="F24" t="str">
+        <v>https://www.dice.com/job-detail/c8cbc56c-9d36-4dfc-b67f-9785ccc187b5</v>
+      </c>
+      <c r="G24" t="str">
+        <v>FP&amp;A</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Easy Apply</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Nextgen Information Services</v>
+      </c>
+      <c r="C25" t="str">
         <v>$50 - $60</v>
       </c>
-      <c r="D16" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-      <c r="F16" t="str">
+      <c r="D25" t="str">
+        <v>Hybrid in Des Peres, Missouri</v>
+      </c>
+      <c r="E25" t="str">
+        <v>9d ago</v>
+      </c>
+      <c r="F25" t="str">
         <v>https://www.dice.com/job-detail/42a6de77-dbb0-45be-b713-9758d2f6ec75</v>
       </c>
-      <c r="G16" t="str">
+      <c r="G25" t="str">
+        <v>FP&amp;A</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Senior Financial Analyst FP&amp;A &amp; Pricing</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Nextgen Information Services</v>
+      </c>
+      <c r="C26" t="str">
+        <v>$50 - $60</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Hybrid in Des Peres, Missouri</v>
+      </c>
+      <c r="E26" t="str">
+        <v>9d ago</v>
+      </c>
+      <c r="F26" t="str">
+        <v>https://www.dice.com/job-detail/42a6de77-dbb0-45be-b713-9758d2f6ec75</v>
+      </c>
+      <c r="G26" t="str">
+        <v>FP&amp;A</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>FP&amp;A Manager</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Judge Group, Inc.</v>
+      </c>
+      <c r="C27" t="str">
+        <v>$150,000</v>
+      </c>
+      <c r="D27" t="str">
+        <v>North Charleston, South Carolina</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Today</v>
+      </c>
+      <c r="F27" t="str">
+        <v>https://www.dice.com/job-detail/6a8561f0-d525-45be-aa81-0e4980ca3449</v>
+      </c>
+      <c r="G27" t="str">
+        <v>FP&amp;A</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Easy Apply</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Ecloud Labs</v>
+      </c>
+      <c r="C28" t="str">
+        <v>000 - 220</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Hybrid in Dallas, Texas</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Yesterday</v>
+      </c>
+      <c r="F28" t="str">
+        <v>https://www.dice.com/job-detail/04db61f5-2a44-4255-b07e-1aeaba956cb9</v>
+      </c>
+      <c r="G28" t="str">
         <v>FP&amp;A</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>